<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-05 Le seau tiède du jardin
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-05.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-05.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le haricot sous la buée</t>
+          <t>Le seau tiède du jardin</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, châssis, thym</t>
+          <t>jardin, tomates vertes, abeille, romarin, thym, seau bleu tiède, pots, terre</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut planter un haricot sous le châssis embué. Raphaël parle peu. Elle lui tend la petite pelle. Ils font un trou. Le haricot disparaît sous la terre tiède.</t>
+          <t>Une goutte tiède pend au romarin. Sur une feuille, un éclat de romarin brille. Nina veut le seau, maintenant. Raphaël ne dit rien. Elle pousse trop vite, eau. Sourire parti, poitrine, papa accroupi. Elle refuse de foncer, tend le seau, attend. Merci vécu. 2e ruse, Dis-le. Un éclat de romarin tient près des tomates.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La vitre du châssis est toute embuée. Un doigt y a dessiné un petit rond. Ça sent le thym et la terre chaude. Une abeille passe près du romarin. Les pots sont encore humides. Papa arrose les pots. L'eau fait un bruit fin. Maman pose un chapeau de paille. Le chapeau sent le soleil. Tu as vu le rond, Nina ? Il est sur la buée. Le thym sent fort, hein ? Oui, maman. Je veux planter un haricot. Sous le châssis. Un haricot à lui, tout seul ? Oui. Dans un petit trou. En ce moment, Nina s'agenouille. La petite pelle est lisse. Le haricot est dans sa poche. Il fait un petit bruit. Raphaël est déjà là. Il parle peu. Il regarde une coccinelle sur le rebord. La coccinelle est rouge et ronde. Nina a envie de tout expliquer. On peut attendre. Tu peux tendre un jouet. Nina tient la petite pelle. Raphaël ne dit rien.</t>
+          <t>Une goutte tiède pend au romarin. Elle tremble, puis tient. Elle est chaude, papa. Tu la vois, Nina ? Oui, papa. Les tomates sont vertes, sous les feuilles. Elles sont dures, maman. Tu les as touchées, Nina ? Oui, maman. Sur une feuille, un éclat de romarin brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Ça sent le thym, tout près. Ça pique le nez. Le thym est fort, Nina ? Oui, maman. Une abeille passe près des tomates. Elle fait un bruit, papa. Près des fleurs ? Oui, tout près. Le seau bleu attend au bord de la terre. Le plastique est tiède, contre la paume. Il est chaud, maman. Tu le tiens, Nina ? Oui. En ce moment, Nina pose le seau. Je veux le seau, maintenant ! Pour les tomates, tout de suite. De l'eau, là ? Oui, de l'eau. Le seau bleu est plein ? Presque. Raphaël arrive près des pots. Il marche sans bruit. Tu verses avec moi ? Raphaël ne dit rien. Il regarde ses mains. Nina a envie de tout expliquer. Les mots montent très vite. Le seau ! L'eau ! Les tomates ! Nina pousse trop vite vers lui. Le seau penche. L'eau tombe sur la terre. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Raphaël, Nina ? Oui, papa. Tes mains tiennent le seau, Nina ? Un peu, maman. L'éclat de romarin tremble, puis tient. Raphaël reste près des pots. Il ne dit rien, papa. Nina regarde papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La vitre du châssis est toute embuée. Un doigt y a dessiné un petit rond. Ça sent le thym et la terre chaude. Une abeille passe près du romarin. Les pots sont encore humides. Papa arrose les pots. L'eau fait un bruit fin. Maman pose un chapeau de paille. Le chapeau sent le soleil. Tu as vu le rond, Nina ? Il est sur la buée. Le thym sent fort, hein ? Oui, maman. Je veux planter un haricot. Sous le châssis. Un haricot à lui, tout seul ? Oui. Dans un petit trou. En ce moment, Nina s'agenouille. La petite pelle est lisse. Le haricot est dans sa poche. Il fait un petit bruit. Raphaël est déjà là. Il parle peu. Il regarde une coccinelle sur le rebord. La coccinelle est rouge et ronde. Nina a envie de tout expliquer. On peut attendre. Tu peux tendre un jouet. Nina tient la petite pelle. Raphaël ne dit rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte tiède pend au romarin. Elle tremble, puis tient. Elle est chaude, papa. Tu la vois, Nina ? Oui, papa. Les tomates sont vertes, sous les feuilles. Elles sont dures, maman. Tu les as touchées, Nina ? Oui, maman. Sur une feuille, un &lt;emphasis level="moderate"&gt;éclat de romarin&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Ça sent le thym, tout près. Ça pique le nez. Le thym est fort, Nina ? Oui, maman. Une abeille passe près des tomates. Elle fait un bruit, papa. Près des fleurs ? Oui, tout près. Le seau bleu attend au bord de la terre. Le plastique est tiède, contre la paume. Il est chaud, maman. Tu le tiens, Nina ? Oui. En ce moment, Nina pose le seau. Je veux le seau, maintenant ! Pour les tomates, tout de suite. De l'eau, là ? Oui, de l'eau. Le seau bleu est plein ? Presque. Raphaël arrive près des pots. Il marche sans bruit. Tu verses avec moi ? Raphaël ne dit rien. Il regarde ses mains. Nina a envie de tout expliquer. Les mots montent très vite. Le seau ! L'eau ! Les tomates ! Nina pousse trop vite vers lui. Le seau penche. L'eau tombe sur la terre. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Raphaël, Nina ? Oui, papa. Tes mains tiennent le seau, Nina ? Un peu, maman. L'éclat de romarin tremble, puis tient. Raphaël reste près des pots. Il ne dit rien, papa. Nina regarde papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Faustine est au jardin avec maman. Marceau est près du bac. Il parle peu. Faustine veut jouer. Maman dit : on peut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. On n'imite pas. On peut tendre un jouet. On ne force pas la parole. Faustine tend le seau. Elle attend. Marceau touche le seau. Il ne dit rien. Faustine sourit. Elle ne force pas la parole. Plus tard, Marceau dit : sable. [pause]</t>
+          <t>Une goutte tiède pend au romarin. Elle tremble, puis tient. Elle est chaude, papa. Tu la vois, Nina ? Oui, papa. Les tomates sont vertes, sous les feuilles. Elles sont dures, maman. Tu les as touchées, Nina ? Oui, maman. Sur une feuille, un &lt;emphasis&gt;éclat de romarin&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Ça sent le thym, tout près. Ça pique le nez. Le thym est fort, Nina ? Oui, maman. Une abeille passe près des tomates. Elle fait un bruit, papa. Près des fleurs ? Oui, tout près. Le seau bleu attend au bord de la terre. Le plastique est tiède, contre la paume. Il est chaud, maman. Tu le tiens, Nina ? Oui. En ce moment, Nina pose le seau. Je veux le seau, maintenant ! Pour les tomates, tout de suite. De l'eau, là ? Oui, de l'eau. Le seau bleu est plein ? Presque. Raphaël arrive près des pots. Il marche sans bruit. Tu verses avec moi ? Raphaël ne dit rien. Il regarde ses mains. Nina a envie de tout expliquer. Les mots montent très vite. Le seau ! L'eau ! Les tomates ! Nina pousse trop vite vers lui. Le seau penche. L'eau tombe sur la terre. Oh. Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Raphaël, Nina ? Oui, papa. Tes mains tiennent le seau, Nina ? Un peu, maman. L'éclat de romarin tremble, puis tient. Raphaël reste près des pots. Il ne dit rien, papa. Nina regarde papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de romarin</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,40 +1326,77 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_seau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La vitre du châssis est toute embuée.
-narrateur|Un doigt y a dessiné un petit rond.
-narrateur|Ça sent le thym et la terre chaude.
-narrateur|Une abeille passe près du romarin.
-narrateur|Les pots sont encore humides.
-narrateur|Papa arrose les pots.
-narrateur|L'eau fait un bruit fin.
-narrateur|Maman pose un chapeau de paille.
-narrateur|Le chapeau sent le soleil.
-papa|Tu as vu le rond, Nina ?
-enfant-f|Il est sur la buée.
-maman|Le thym sent fort, hein ?
+          <t>narrateur|Une goutte tiède pend au romarin.
+narrateur|Elle tremble, puis tient.
+enfant-f|Elle est chaude, papa.
+papa|Tu la vois, Nina ?
+enfant-f|Oui, papa.
+narrateur|Les tomates sont vertes, sous les feuilles.
+enfant-f|Elles sont dures, maman.
+maman|Tu les as touchées, Nina ?
 enfant-f|Oui, maman.
-enfant-f|Je veux planter un haricot.
-enfant-f|Sous le châssis.
-papa|Un haricot à lui, tout seul ?
+narrateur|Sur une feuille, un éclat de romarin brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Ça sent le thym, tout près.
+enfant-f|Ça pique le nez.
+maman|Le thym est fort, Nina ?
+enfant-f|Oui, maman.
+narrateur|Une abeille passe près des tomates.
+enfant-f|Elle fait un bruit, papa.
+papa|Près des fleurs ?
+enfant-f|Oui, tout près.
+narrateur|Le seau bleu attend au bord de la terre.
+narrateur|Le plastique est tiède, contre la paume.
+enfant-f|Il est chaud, maman.
+maman|Tu le tiens, Nina ?
 enfant-f|Oui.
-enfant-f|Dans un petit trou.
-narrateur|En ce moment, Nina s'agenouille.
-narrateur|La petite pelle est lisse.
-narrateur|Le haricot est dans sa poche.
-narrateur|Il fait un petit bruit.
-narrateur|Raphaël est déjà là.
-narrateur|Il parle peu.
-narrateur|Il regarde une coccinelle sur le rebord.
-narrateur|La coccinelle est rouge et ronde.
+narrateur|En ce moment, Nina pose le seau.
+enfant-f|Je veux le seau, maintenant !
+enfant-f|Pour les tomates, tout de suite.
+papa|De l'eau, là ?
+enfant-f|Oui, de l'eau.
+maman|Le seau bleu est plein ?
+enfant-f|Presque.
+narrateur|Raphaël arrive près des pots.
+narrateur|Il marche sans bruit.
+enfant-f|Tu verses avec moi ?
+narrateur|Raphaël ne dit rien.
+narrateur|Il regarde ses mains.
 narrateur|Nina a envie de tout expliquer.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
-narrateur|Nina tient la petite pelle.
-narrateur|Raphaël ne dit rien.</t>
+narrateur|Les mots montent très vite.
+enfant-f|Le seau !
+enfant-f|L'eau !
+enfant-f|Les tomates !
+narrateur|Nina pousse trop vite vers lui.
+narrateur|Le seau penche.
+narrateur|L'eau tombe sur la terre.
+enfant-f|Oh.
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Raphaël, Nina ?
+enfant-f|Oui, papa.
+maman|Tes mains tiennent le seau, Nina ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de romarin tremble, puis tient.
+narrateur|Raphaël reste près des pots.
+enfant-f|Il ne dit rien, papa.
+narrateur|Nina regarde papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>jardin,eau</t>
         </is>
       </c>
     </row>
@@ -1391,12 +1428,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël parle peu. Que fait Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël parle peu. Que fait &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Marceau parle peu. Que fait Faustine ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël parle peu. Que fait &lt;emphasis&gt;Nina&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1406,7 +1443,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>attendre | tendre | la pelle | un jouet | elle attend</t>
+          <t>attendre | tendre | le seau | un jouet</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1459,7 +1496,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1470,7 +1507,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1485,34 +1522,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1527,17 +1568,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=raphael_parle_peu_que_fait_nina; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1570,17 +1611,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina tend la petite pelle. Pour le trou. Elle attend. Un grain de terre colle à son genou. Raphaël touche la pelle. Il ne dit rien. On ne force pas la parole. La terre n'a pas besoin de mots. Raphaël prend la pelle. Il creuse près du thym. Nina pose le haricot. Il est lisse et un peu froid. Raphaël recouvre. La terre est tiède. Elle sent le jardin. Un peu l'eau. Un peu le thym. Il est caché. Puis Raphaël dit tout bas. Haricot. Haricot. Tu as su attendre. Bravo, Nina. Papa verse un peu d'eau. La terre devient sombre. Une petite flaque brille, puis s'en va.</t>
+          <t>Nina veut le seau, tout de suite. Prends-le, maintenant ! Elle avance trop vite vers Raphaël. Les mots se bousculent dans sa bouche. Raphaël recule un peu. Il serre les mains contre lui. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le seau, un instant. Elle écoute l'abeille près des feuilles. Tu veux l'eau avec Raphaël ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le seau, puis on reste. D'accord. Nina reste un moment, les mains ouvertes. Elle attend. Elle tend le seau. Pour toi. Raphaël ne dit rien. Il prend le seau, sans parler. Oui. Nina pose les mains sur la terre. Elle reste, sans se presser. Raphaël tient le seau, plus lentement. Merci, Nina. Papa a vu les deux, au jardin. Le plastique est tiède, sous les doigts. Il est chaud. Un peu d'eau reste au fond. Le seau. Il a de l'eau, là ? Oui, là. Nina glisse la main sur le bord. Le plastique est doux, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Raphaël s'assoit, puis se relève. Seau. On va jusqu'aux tomates ? Les tomates vertes sont près du thym. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina tend la petite pelle. Pour le trou. Elle attend. Un grain de terre colle à son genou. Raphaël touche la pelle. Il ne dit rien. On ne force pas la parole. La terre n'a pas besoin de mots. Raphaël prend la pelle. Il creuse près du thym. Nina pose le haricot. Il est lisse et un peu froid. Raphaël recouvre. La terre est tiède. Elle sent le jardin. Un peu l'eau. Un peu le thym. Il est caché. Puis Raphaël dit tout bas. Haricot. Haricot. Tu as su attendre. Bravo, Nina. Papa verse un peu d'eau. La terre devient sombre. Une petite flaque brille, puis s'en va.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, tout de suite. Prends-le, maintenant ! Elle avance trop vite vers Raphaël. Les mots se bousculent dans sa bouche. Raphaël recule un peu. Il serre les mains contre lui. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le seau, un instant. Elle écoute l'abeille près des feuilles. Tu veux l'eau avec Raphaël ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le seau, puis on reste. D'accord. Nina reste un moment, les mains ouvertes. Elle attend. Elle tend le seau. Pour toi. Raphaël ne dit rien. Il prend le seau, sans parler. Oui. Nina pose les mains sur la terre. Elle reste, sans se presser. Raphaël tient le seau, plus lentement. Merci, Nina. Papa a vu les deux, au jardin. Le plastique est tiède, sous les doigts. Il est chaud. Un peu d'eau reste au fond. Le seau. Il a de l'eau, là ? Oui, là. Nina glisse la main sur le bord. Le plastique est doux, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Raphaël s'assoit, puis se relève. Seau. On va jusqu'aux tomates ? Les tomates vertes sont près du thym. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Faustine a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Elle a tendu un jouet. Elle n'a pas forcé la parole. [pause]</t>
+          <t>Nina veut le &lt;emphasis&gt;seau&lt;/emphasis&gt;, tout de suite. Prends-le, maintenant ! Elle avance trop vite vers Raphaël. Les mots se bousculent dans sa bouche. Raphaël recule un peu. Il serre les mains contre lui. Oh. Le sourire ne revient pas. Nina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le seau, un instant. Elle écoute l'abeille près des feuilles. Tu veux l'eau avec Raphaël ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le seau, puis on reste. D'accord. Nina reste un moment, les mains ouvertes. Elle attend. Elle tend le seau. Pour toi. Raphaël ne dit rien. Il prend le seau, sans parler. Oui. Nina pose les mains sur la terre. Elle reste, sans se presser. Raphaël tient le seau, plus lentement. Merci, Nina. Papa a vu les deux, au jardin. Le plastique est tiède, sous les doigts. Il est chaud. Un peu d'eau reste au fond. Le seau. Il a de l'eau, là ? Oui, là. Nina glisse la main sur le bord. Le plastique est doux, contre la peau. Tes mains sont au chaud, Nina ? Un peu, maman. Raphaël s'assoit, puis se relève. Seau. On va jusqu'aux tomates ? Les tomates vertes sont près du thym. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1627,7 +1668,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1635,10 +1676,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1661,30 +1702,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1693,10 +1734,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1709,37 +1750,61 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_tend_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina tend la petite pelle.
-enfant-f|Pour le trou.
+          <t>narrateur|Nina veut le seau, tout de suite.
+enfant-f|Prends-le, maintenant !
+narrateur|Elle avance trop vite vers Raphaël.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Raphaël recule un peu.
+narrateur|Il serre les mains contre lui.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le seau, un instant.
+narrateur|Elle écoute l'abeille près des feuilles.
+papa|Tu veux l'eau avec Raphaël ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Papa, on fait quoi ?
+papa|On pose le seau, puis on reste.
+enfant-f|D'accord.
+narrateur|Nina reste un moment, les mains ouvertes.
 narrateur|Elle attend.
-narrateur|Un grain de terre colle à son genou.
-narrateur|Raphaël touche la pelle.
-narrateur|Il ne dit rien.
-maman|On ne force pas la parole.
-papa|La terre n'a pas besoin de mots.
-narrateur|Raphaël prend la pelle.
-narrateur|Il creuse près du thym.
-narrateur|Nina pose le haricot.
-narrateur|Il est lisse et un peu froid.
-narrateur|Raphaël recouvre.
-narrateur|La terre est tiède.
-narrateur|Elle sent le jardin.
-narrateur|Un peu l'eau.
-narrateur|Un peu le thym.
-enfant-f|Il est caché.
-narrateur|Puis Raphaël dit tout bas.
-enfant-m|Haricot.
-enfant-f|Haricot.
-papa|Tu as su attendre.
-papa|Bravo, Nina.
-narrateur|Papa verse un peu d'eau.
-narrateur|La terre devient sombre.
-narrateur|Une petite flaque brille, puis s'en va.</t>
+narrateur|Elle tend le seau.
+enfant-f|Pour toi.
+narrateur|Raphaël ne dit rien.
+narrateur|Il prend le seau, sans parler.
+copain|Oui.
+narrateur|Nina pose les mains sur la terre.
+narrateur|Elle reste, sans se presser.
+narrateur|Raphaël tient le seau, plus lentement.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux, au jardin.
+maman|Le plastique est tiède, sous les doigts.
+enfant-f|Il est chaud.
+narrateur|Un peu d'eau reste au fond.
+enfant-f|Le seau.
+papa|Il a de l'eau, là ?
+enfant-f|Oui, là.
+narrateur|Nina glisse la main sur le bord.
+narrateur|Le plastique est doux, contre la peau.
+maman|Tes mains sont au chaud, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Raphaël s'assoit, puis se relève.
+copain|Seau.
+enfant-f|On va jusqu'aux tomates ?
+maman|Les tomates vertes sont près du thym.
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>seau,eau</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1831,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman essuie un peu la buée. Le rond a disparu. On voit le haricot caché, presque. Un peu d'eau, pour toi ? Raphaël secoue la tête. D'accord. D'accord. Tu as fini le trou, Nina ? Oui, maman. Le haricot est dessous. Papa ferme le robinet. L'eau s'arrête. Nina donne la main. Le chapeau de paille reste sur le banc. La coccinelle s'en va. Le thym sent encore. L'abeille s'éloigne. Le thym reste. Oui. Il sent encore.</t>
+          <t>Ils restent près des tomates. Le seau bleu penche vers une feuille. Je verse, maintenant ! Nina pousse trop vite. L'eau gicle sur le pied de Raphaël. Ça mouille ! Dis-le, Raphaël ! Raphaël serre les lèvres. Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le thym, tout près. Près des feuilles, un éclat de romarin luit. Là, sur le romarin. Tu prends le seau, Raphaël ? Raphaël ne dit rien. Il tend les mains, sans parler. Oui. Nina passe le seau, sans se presser. Raphaël le reçoit, plus lentement. Le plastique est lisse et tiède. Tu le vois, le seau ? Oui, papa. L'eau est tiède, Nina ? Oui, maman. Raphaël verse, un filet mince. La terre devient sombre, sous les tomates. La terre boit, Nina ? Oui, papa. Un rayon passe sur le romarin. Il allume la feuille.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman essuie un peu la buée. Le rond a disparu. On voit le haricot caché, presque. Un peu d'eau, pour toi ? Raphaël secoue la tête. D'accord. D'accord. Tu as fini le trou, Nina ? Oui, maman. Le haricot est dessous. Papa ferme le robinet. L'eau s'arrête. Nina donne la main. Le chapeau de paille reste sur le banc. La coccinelle s'en va. Le thym sent encore. L'abeille s'éloigne. Le thym reste. Oui. Il sent encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent près des tomates. Le seau bleu penche vers une feuille. Je verse, maintenant ! Nina pousse trop vite. L'eau gicle sur le pied de Raphaël. Ça mouille ! Dis-le, Raphaël ! Raphaël serre les lèvres. Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le thym, tout près. Près des feuilles, un &lt;emphasis level="moderate"&gt;éclat de romarin&lt;/emphasis&gt; luit. Là, sur le romarin. Tu prends le seau, Raphaël ? Raphaël ne dit rien. Il tend les mains, sans parler. Oui. Nina passe le seau, sans se presser. Raphaël le reçoit, plus lentement. Le plastique est lisse et tiède. Tu le vois, le seau ? Oui, papa. L'eau est tiède, Nina ? Oui, maman. Raphaël verse, un filet mince. La terre devient sombre, sous les tomates. La terre boit, Nina ? Oui, papa. Un rayon passe sur le romarin. Il allume la feuille.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range le seau. Faustine donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils restent près des tomates. Le seau bleu penche vers une feuille. Je verse, maintenant ! Nina pousse trop vite. L'eau gicle sur le pied de Raphaël. Ça mouille ! Dis-le, Raphaël ! Raphaël serre les lèvres. Nina avance les mains, trop vite. Puis elle s'arrête net. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le seau, un instant. Elle écoute le thym, tout près. Près des feuilles, un &lt;emphasis&gt;éclat de romarin&lt;/emphasis&gt; luit. Là, sur le romarin. Tu prends le seau, Raphaël ? Raphaël ne dit rien. Il tend les mains, sans parler. Oui. Nina passe le seau, sans se presser. Raphaël le reçoit, plus lentement. Le plastique est lisse et tiède. Tu le vois, le seau ? Oui, papa. L'eau est tiède, Nina ? Oui, maman. Raphaël verse, un filet mince. La terre devient sombre, sous les tomates. La terre boit, Nina ? Oui, papa. Un rayon passe sur le romarin. Il allume la feuille. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1888,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,10 +1896,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,30 +1922,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de romarin</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,10 +1954,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1903,29 +1968,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=eau_trop_vite_dis_le_elle_s_arrete; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman essuie un peu la buée.
-narrateur|Le rond a disparu.
-narrateur|On voit le haricot caché, presque.
-maman|Un peu d'eau, pour toi ?
-narrateur|Raphaël secoue la tête.
-enfant-f|D'accord.
-papa|D'accord.
-maman|Tu as fini le trou, Nina ?
+          <t>narrateur|Ils restent près des tomates.
+narrateur|Le seau bleu penche vers une feuille.
+enfant-f|Je verse, maintenant !
+narrateur|Nina pousse trop vite.
+narrateur|L'eau gicle sur le pied de Raphaël.
+enfant-f|Ça mouille !
+enfant-f|Dis-le, Raphaël !
+narrateur|Raphaël serre les lèvres.
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le seau, un instant.
+narrateur|Elle écoute le thym, tout près.
+narrateur|Près des feuilles, un éclat de romarin luit.
+enfant-f|Là, sur le romarin.
+enfant-f|Tu prends le seau, Raphaël ?
+narrateur|Raphaël ne dit rien.
+narrateur|Il tend les mains, sans parler.
+copain|Oui.
+narrateur|Nina passe le seau, sans se presser.
+narrateur|Raphaël le reçoit, plus lentement.
+narrateur|Le plastique est lisse et tiède.
+papa|Tu le vois, le seau ?
+enfant-f|Oui, papa.
+maman|L'eau est tiède, Nina ?
 enfant-f|Oui, maman.
-enfant-f|Le haricot est dessous.
-narrateur|Papa ferme le robinet.
-narrateur|L'eau s'arrête.
-narrateur|Nina donne la main.
-narrateur|Le chapeau de paille reste sur le banc.
-papa|La coccinelle s'en va.
-narrateur|Le thym sent encore.
-narrateur|L'abeille s'éloigne.
-enfant-f|Le thym reste.
-papa|Oui.
-papa|Il sent encore.</t>
+narrateur|Raphaël verse, un filet mince.
+narrateur|La terre devient sombre, sous les tomates.
+papa|La terre boit, Nina ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le romarin.
+enfant-f|Il allume la feuille.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>eau,tomates</t>
         </is>
       </c>
     </row>
@@ -1952,17 +2040,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le haricot est sous la terre. Sous le châssis. Il a de l'eau, maintenant.</t>
+          <t>Ils restent près des tomates. Le seau est vide, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. Le plastique sent bon. Tu le sens, le seau ? Oui, maman. La terre reste un peu, sombre. Elle a bu, sous les tomates. Seau. Le seau bleu fait de l'ombre. L'abeille s'éloigne, sans bruit. On y remet de l'eau, après. Un éclat de romarin tient près des tomates.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le haricot est sous la terre. Sous le châssis. Il a de l'eau, maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près des tomates. Le seau est vide, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. Le plastique sent bon. Tu le sens, le seau ? Oui, maman. La terre reste un peu, sombre. Elle a bu, sous les tomates. Seau. Le seau bleu fait de l'ombre. L'abeille s'éloigne, sans bruit. On y remet de l'eau, après. Un &lt;emphasis level="moderate"&gt;éclat de romarin&lt;/emphasis&gt; tient près des tomates.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près des tomates. Le seau est vide, Nina ? Oui, maman. Tu souffles un peu ? Oui, papa. Nina souffle, un filet d'air. Le plastique sent bon. Tu le sens, le seau ? Oui, maman. La terre reste un peu, sombre. Elle a bu, sous les tomates. Seau. Le seau bleu fait de l'ombre. L'abeille s'éloigne, sans bruit. On y remet de l'eau, après. Un &lt;emphasis&gt;éclat de romarin&lt;/emphasis&gt; tient près des tomates.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2009,15 +2097,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2029,12 +2117,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2043,17 +2131,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de romarin</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2062,11 +2154,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2075,26 +2167,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pres_des_tomates; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Le haricot est sous la terre.
-maman|Sous le châssis.
-papa|Il a de l'eau, maintenant.</t>
+          <t>narrateur|Ils restent près des tomates.
+maman|Le seau est vide, Nina ?
+enfant-f|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-f|Oui, papa.
+narrateur|Nina souffle, un filet d'air.
+enfant-f|Le plastique sent bon.
+maman|Tu le sens, le seau ?
+enfant-f|Oui, maman.
+papa|La terre reste un peu, sombre.
+enfant-f|Elle a bu, sous les tomates.
+copain|Seau.
+narrateur|Le seau bleu fait de l'ombre.
+narrateur|L'abeille s'éloigne, sans bruit.
+enfant-f|On y remet de l'eau, après.
+narrateur|Un éclat de romarin tient près des tomates.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>jardin,romarin</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2172,6 +2286,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>